<commit_message>
finished code for curating data step
</commit_message>
<xml_diff>
--- a/data/LMini_iNat_Pops_filtered_curated_metadata.xlsx
+++ b/data/LMini_iNat_Pops_filtered_curated_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\allen\Documents\R\Data_Sci_Leptosiphon_Polymorphism\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E99A2A2-C504-4F4A-820F-AF11DACEBF66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E51795A6-06C8-4F0C-B508-693CD8D3AD56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2DDA18C5-069F-4AEC-9FB6-1E496F22AE95}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="58">
   <si>
     <t>url</t>
   </si>
@@ -202,6 +202,12 @@
   </si>
   <si>
     <t>pop of ~1000</t>
+  </si>
+  <si>
+    <t>Dist to shore (km)</t>
+  </si>
+  <si>
+    <t>Dist to Mainland (km)</t>
   </si>
 </sst>
 </file>
@@ -1074,15 +1080,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C996E96A-1C90-4402-AD00-F0348FA66D0F}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="4" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="44" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -1116,8 +1126,14 @@
       <c r="K1" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -1143,8 +1159,14 @@
       <c r="H2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L2">
+        <v>0.34</v>
+      </c>
+      <c r="M2">
+        <v>22.75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1170,8 +1192,14 @@
       <c r="H3" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L3">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="M3">
+        <v>6.51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1197,8 +1225,14 @@
       <c r="H4" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L4">
+        <v>1.41</v>
+      </c>
+      <c r="M4">
+        <v>38.68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -1224,8 +1258,14 @@
       <c r="H5" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L5">
+        <v>1.63</v>
+      </c>
+      <c r="M5">
+        <v>32.85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1251,8 +1291,14 @@
       <c r="H6" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L6">
+        <v>0.21</v>
+      </c>
+      <c r="M6">
+        <v>6.25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1279,7 +1325,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1306,7 +1352,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -1332,8 +1378,14 @@
       <c r="H9" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L9">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="M9">
+        <v>6.26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1359,8 +1411,14 @@
       <c r="H10" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L10">
+        <v>0.2</v>
+      </c>
+      <c r="M10">
+        <v>22.62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
@@ -1386,8 +1444,11 @@
       <c r="H11" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L11">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
@@ -1413,8 +1474,11 @@
       <c r="H12" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L12">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
@@ -1441,7 +1505,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>6</v>
       </c>
@@ -1468,7 +1532,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
@@ -1495,7 +1559,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
@@ -1522,7 +1586,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
@@ -1549,7 +1613,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>6</v>
       </c>
@@ -1576,7 +1640,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>6</v>
       </c>
@@ -1603,7 +1667,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>6</v>
       </c>
@@ -1630,7 +1694,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>6</v>
       </c>
@@ -1657,7 +1721,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>6</v>
       </c>
@@ -1684,7 +1748,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>6</v>
       </c>
@@ -1711,7 +1775,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>6</v>
       </c>
@@ -1738,7 +1802,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>6</v>
       </c>
@@ -1765,7 +1829,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>6</v>
       </c>
@@ -1791,8 +1855,11 @@
       <c r="H26" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L26">
+        <v>0.93462999999999996</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>6</v>
       </c>
@@ -1818,8 +1885,11 @@
       <c r="H27" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L27">
+        <v>0.53893000000000002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>6</v>
       </c>
@@ -1849,7 +1919,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>6</v>
       </c>
@@ -1876,7 +1946,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>6</v>
       </c>
@@ -1903,7 +1973,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
@@ -1929,8 +1999,11 @@
       <c r="H31" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L31">
+        <v>0.37801000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>6</v>
       </c>
@@ -1959,8 +2032,11 @@
       <c r="I32" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L32">
+        <v>1.746E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>6</v>
       </c>
@@ -1986,8 +2062,11 @@
       <c r="H33" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L33">
+        <v>1.7294499999999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>6</v>
       </c>
@@ -2016,8 +2095,11 @@
       <c r="I34" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L34">
+        <v>1.09E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>6</v>
       </c>
@@ -2045,6 +2127,9 @@
       </c>
       <c r="I35" t="s">
         <v>53</v>
+      </c>
+      <c r="L35">
+        <v>9.9299999999999996E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>